<commit_message>
Rewrite Mode 3 Golden Path doc for the new native-MO cutting mechanism
Yesterday's Session 129/ADR-061 tore down Factory Worklist and the
Cut-to-Order/Request Material wizards entirely, replacing them with a
plain native Manufacturing Order (Admin picks the Block directly, no
wizard). The old doc's entire case list described buttons/menus that no
longer exist, so this is a full case-list rewrite, not a screenshot
refresh -- also the first real live Playwright click-through of the new
mechanism's SO-linked path (auto-hold + price recalc on Complete Cut).
Fresh fixture: PO P00053 -> BLK-26-0028 -> SO S00125 -> MO
EG01/STCUT/00042 -> Delivery EG01/OUT/00079 -> INV/2026/00027.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode3.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode3.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="F1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="F2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="F3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="F4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="E1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="E2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="E3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="E4" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,14 +484,14 @@
     <row r="5">
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Total test cases: 14</t>
+          <t>Total test cases: 13</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 9 / 5 / 0</t>
+          <t>High / Medium / Low: 11 / 2 / 0</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
     <row r="9">
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>F1 — ขาย (Sale — Mode 3, Cut-to-Order)</t>
+          <t>E1 — ขาย (Sale — ก่อนมีแผ่นจริง)</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -520,17 +520,17 @@
     <row r="10">
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>F2 — การผลิต (Production — Factory Worklist / Request Material / Cut Order)</t>
+          <t>E2 — ผลิต (Production — ตัด Slab จริง)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>F3 — จัดส่ง (Delivery — Scan Verification)</t>
+          <t>E3 — จัดส่ง (Delivery — Scan Verification)</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -540,7 +540,7 @@
     <row r="12">
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>F4 — บัญชี (Accounting + Payment)</t>
+          <t>E4 — บัญชี (Accounting + Payment)</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -578,7 +578,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F1. ขาย (Sale — Mode 3, Cut-to-Order) — ADR-018 — ยืนยันคำสั่งขายได้ทันทีแม้ยังไม่มีแผ่นหินจริง</t>
+          <t>E1. ขาย (Sale — ก่อนมีแผ่นจริง) — ADR-018 — ขายได้ทันทีแม้ยังไม่มีแผ่น ราคาจะคำนวณจริงหลังตัดเสร็จ</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>เพิ่มบรรทัดสินค้า Material โหมด Cut-to-Order ใน Sale Order</t>
+          <t>เพิ่มบรรทัดสินค้า Material ที่ยังไม่มีแผ่นจริงในสต็อก</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>มี Block พร้อมอยู่แล้วในสต็อกของ Material นี้ (Pricing Mode = Serial) แต่ยังไม่มีแผ่นสำเร็จรูปขนาดที่ลูกค้าต้องการอยู่ในสต็อก</t>
+          <t>มี Block พร้อมอยู่แล้วในสต็อก (ยังไม่ตัด) จาก Material ที่ตั้ง Pricing Mode = Serial (per-slab)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -670,12 +670,12 @@
       <c r="E4" s="7" t="inlineStr">
         <is>
           <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
-สินค้า = "Rosso Levanto Test - Slab"</t>
+สินค้า = E2E Mode3 Fresh Test - Slab</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เพิ่มบรรทัดสำเร็จ ราคาต่อหน่วยขึ้นเป็นราคาตั้งต้นของสินค้า (list price) เนื่องจากยังไม่มีแผ่นจริงผูกกับบรรทัดนี้เลย</t>
+          <t>เพิ่มบรรทัดสำเร็จ ราคาต่อหน่วยขึ้นเป็นราคาตั้งต้นของสินค้า (list price) เนื่องจากยังไม่มีแผ่นจริงผูกกับบรรทัดนี้เลย (ตัวอย่างจริง: 4,500/หน่วย)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>ยืนยัน (Confirm) Sale Order ได้ทันที โดยยังไม่ทราบขนาดที่จะตัด</t>
+          <t>ยืนยัน (Confirm) Sale Order ทั้งที่ยังไม่มีแผ่นจริง</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น Sales Order ยอดรวมคำนวณจากราคาตั้งต้นของสินค้า (ตัวอย่างจริง: S00095, 4,500 + VAT 7% = 4,815.00 บาท) — ราคานี้ยังไม่ใช่ราคาจริง จะคำนวณใหม่อัตโนมัติหลังฝ่ายผลิตตัดแผ่นเสร็จ (ดู TC-E2E-M3-08) มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ</t>
+          <t>SO เปลี่ยนสถานะเป็น Sales Order ยอดรวมคำนวณจากราคาตั้งต้นของสินค้า (ตัวอย่างจริง: S00125, 4,500 + VAT 7% = 4,815.00 บาท) — ราคานี้ยังไม่ใช่ราคาจริง จะคำนวณใหม่อัตโนมัติหลังตัดเสร็จ (ดู TC-E2E-M3-07) มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ แต่ยังส่งไม่ได้เพราะยังไม่มีของจริง</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -765,7 +765,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F2. การผลิต (Production — Factory Worklist / Request Material / Cut Order) — ADR-018 + ADR-053 — ย้าย Block ไปสถานีตัดก่อนเสมอ ก่อนสร้างใบสั่งผลิตได้</t>
+          <t>E2. ผลิต (Production — ตัด Slab จริง) — กลไกใหม่ 13 ก.ย. 2026 — สร้าง Manufacturing Order ตรงในแอป Manufacturing ไม่ต้องผ่าน wizard แล้ว</t>
         </is>
       </c>
     </row>
@@ -839,35 +839,45 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>เห็นคิวงานที่หน้า Factory Worklist</t>
+          <t>สร้าง Manufacturing Order ผูกกับ Block และ SO line โดยตรง</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-02 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M3-02 เสร็จแล้ว มี Block พร้อมอยู่แล้วในสต็อก (ยังไม่ตัด)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดเมนู Factory Worklist</t>
+          <t>1. เปิด Manufacturing &gt; New
+2. เลือก "Stone Block" เป็น Block ที่ต้องการตัด
+3. กรอก "Target Slab L (M)" และ "Target Slab H (M)"
+4. เลือก "For Sale Order Line" ผูกกับบรรทัด SO ที่รอแผ่นอยู่</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Stone Block = BLK-26-0028
+Target Slab L (M) = 1.2
+Target Slab H (M) = 0.8
+For Sale Order Line = S00125</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เห็นแถวของ SO นี้ขึ้นคิวงาน ช่อง "ต้องทำ" ระบุ "รอเลือก/ตัด Slab (Cut to Order)" คอลัมน์ "ความพร้อม Block" ขึ้นเตือน (ยังไม่พร้อมตัด — ต้องย้าย Block ก่อน)</t>
+          <t>สร้าง Manufacturing Order สำเร็จ ระบบเติม Product และ Bill of Material ให้อัตโนมัติจาก Block ที่เลือก (ตัวอย่างจริง: EG01/STCUT/00042)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="n"/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>✨ กลไกใหม่ (เปลี่ยน 13 ก.ย. 2026): ไม่มี "Factory Worklist"/"Cut to Order" wizard แล้ว — Admin สร้าง Manufacturing Order ตรงในแอป Manufacturing ได้เลย เลือก Block ที่ช่อง "Stone Block" ระบบจะเติม Product/Bill of Material ให้อัตโนมัติ</t>
+        </is>
+      </c>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
@@ -881,7 +891,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>พยายามกด "Cut to Order" ก่อนย้าย Block ไปสถานีตัด</t>
+          <t>พยายาม Confirm Manufacturing Order โดย Block ยังไม่ได้ย้ายไปสถานีตัด</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -891,20 +901,17 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม "Cut to Order" บนแถวนั้น
-2. เลือกก้อนหินที่จะตัด กรอกขนาดที่จะตัด
-3. กด "Create Cut Order"</t>
+          <t>1. กดปุ่ม Confirm บน Manufacturing Order ทันที</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Block = BLK-26-0013
-ขนาดที่จะตัด = 1.2 × 0.8 ม.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ระบบฟ้อง error สองภาษาทันที ระบุปริมาณที่ต้องการเทียบกับที่มีอยู่จริงที่สถานีตัด บันทึกไม่ผ่าน — ตัวอย่างจริง: "Block BLK-26-0013 ยังไม่ได้ย้ายไปสถานีตัด (Stone Production) เพียงพอ — ต้องการ 0.019 m³ แต่อยู่ที่สถานีตัดแล้วแค่ 0.000 m³"</t>
+          <t>ระบบฟ้อง error สองภาษาทันที ระบุปริมาณที่ต้องการเทียบกับที่มีอยู่จริงที่สถานีตัด บันทึกไม่ผ่าน — ตัวอย่างจริง: "Block BLK-26-0028 ยังไม่ได้ย้ายไปสถานีตัด (Stone Production) เพียงพอ — ต้องการ 0.019 m³ แต่อยู่ที่สถานีตัดแล้วแค่ 0.000 m³"</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -912,11 +919,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>หมายเหตุ: กันตัดจากก้อนที่ยังไม่ได้อยู่หน้างานจริง (ADR-053) — จำลองขั้นตอนหน้างานจริงที่ต้องยกก้อนหินไปวางที่แท่นตัดก่อนเริ่มงาน</t>
-        </is>
-      </c>
+      <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
@@ -930,7 +933,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>กด "Request Material" ขอย้าย Block ไปสถานีตัด</t>
+          <t>ย้าย Block ไปสถานีตัด (Internal Transfer)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -940,21 +943,21 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. กลับไปที่ Factory Worklist กดปุ่ม "Request Material" บนแถวเดิม
-2. กรอกขนาด/ความหนาเป้าหมายที่จะตัด
-3. กด "Request Material" ยืนยัน</t>
+          <t>1. เปิด Inventory &gt; Internal Transfers &gt; New
+2. Source Location = Stone Available, Destination Location = Stone Production
+3. เพิ่มสินค้า Block นั้น กรอกจำนวนที่ต้องการย้าย
+4. กด Validate</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Target L = 1.2 ม.
-Target H = 0.8 ม.
-Target Thickness = 0.02 ม.</t>
+          <t>สินค้า = E2E Mode3 Fresh Test - Block
+จำนวน = 0.02 m³</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ระบบสร้างใบขอย้ายสินค้า (Internal Transfer) อัตโนมัติ 1 ใบ ปลายทาง "Stone Production" — ตัวอย่างจริง: EG01/STPR/00009 (0.0192 m³)</t>
+          <t>ใบย้ายสถานะเปลี่ยนเป็น Done สำเร็จ — ตัวอย่างจริง: EG01/INT/00058 — Block ก้อนนั้นย้ายไปอยู่ที่ Location "Stone Production" ครบตามจำนวนที่ย้าย</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -976,29 +979,28 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>(ฝ่ายคลัง) ยืนยันใบขอย้าย — ระบุก้อนหินจริงที่จะใช้แล้ว Validate</t>
+          <t>กลับไป Confirm Manufacturing Order อีกครั้ง</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-05 เสร็จแล้ว มีใบขอย้ายสถานะรออยู่</t>
+          <t>ทำ TC-E2E-M3-05 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบขอย้ายที่เกิดขึ้น
-2. ระบุ/สแกนก้อนหิน (Lot) ที่จะใช้จริงพร้อมจำนวน
-3. กด Validate</t>
+          <t>1. กลับไปที่ Manufacturing Order เดิม
+2. กดปุ่ม Confirm อีกครั้ง</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Lot = BLK-26-0013-BLK</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ใบขอย้ายเปลี่ยนสถานะเป็น Done ก้อนหินย้ายไปอยู่ที่ Location "Stone Production" ครบตามจำนวนที่ขอ</t>
+          <t>ยืนยันสำเร็จ ไม่มี error แล้ว เพราะ Block ถูกย้ายมาสถานีตัดครบตามจำนวนแล้ว — สถานะเปลี่ยนเป็น Confirmed ปุ่ม "Complete Cut" ปรากฏพร้อมกดขั้นถัดไป</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1006,11 +1008,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>เช่นเดียวกับ Barcode app จริง: ระบบยังไม่เลือกก้อนหินให้ล่วงหน้า ฝ่ายคลังเป็นผู้ระบุว่าจะใช้ก้อนไหนตอนย้ายจริง (ADR-053)</t>
-        </is>
-      </c>
+      <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
@@ -1024,7 +1022,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>กด "Cut to Order" อีกครั้ง — สร้างใบสั่งผลิตสำเร็จ</t>
+          <t>กด "Complete Cut" — ได้แผ่นจริง ราคา SO คำนวณใหม่อัตโนมัติ</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1034,20 +1032,18 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>1. กลับไปที่ Factory Worklist กดปุ่ม "Cut to Order" อีกครั้ง
-2. เลือกก้อนหินเดิม กรอกขนาดเดิม
-3. กด "Create Cut Order"</t>
+          <t>1. กดปุ่ม "Complete Cut" บน Manufacturing Order
+2. กลับไปเปิด Sale Order เดิมดูราคา</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Block = BLK-26-0013
-ขนาดที่จะตัด = 1.2 × 0.8 ม.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>สร้างใบสั่งผลิต (Manufacturing Order) สำเร็จ ไม่มี error แล้ว เพราะ Block ถูกย้ายมาสถานีตัดครบตามจำนวนแล้ว — ตัวอย่างจริง: EG01/STCUT/00036</t>
+          <t>Manufacturing Order เสร็จสมบูรณ์ (สถานะ Done) เกิดแผ่นหินใหม่ 1 แผ่นตามขนาดที่ตัดจริง (Lot/Serial ใหม่) ผูกกับบรรทัด SO เดิมให้อัตโนมัติ ราคาต่อหน่วยของบรรทัด SO เปลี่ยนจากราคาตั้งต้นเป็นราคาจริงตามขนาดที่ตัดได้ทันที — ตัวอย่างจริง: แผ่น BLK-26-0028-1 (1.2×0.8 ม. = 0.96 ตร.ม.) ยอดรวม SO เปลี่ยนจาก 4,815.00 เป็น 4,622.40 (รวม VAT) ทันที เห็นการเปลี่ยนแปลงบันทึกไว้ใน chatter log ของ SO</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1060,49 +1056,6 @@
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M3-08</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>ตัดแผ่นเสร็จ (Mark Done) — ราคาคำนวณใหม่อัตโนมัติ</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M3-07 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิดใบสั่งผลิต
-2. กดปุ่มยืนยันตัดเสร็จ (Mark Done)</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>ใบสั่งผลิตเสร็จสมบูรณ์ เกิดแผ่นหินใหม่ 1 แผ่นตามขนาดที่ตัดจริง ผูกกับบรรทัด SO เดิมให้อัตโนมัติ ราคาต่อหน่วยของบรรทัด SO เปลี่ยนจากราคาตั้งต้นเป็นราคาจริงตามขนาดที่ตัดได้ — ตัวอย่างจริง: แผ่น BLK-26-0013 #2 (1.2×0.8 ม.) ราคา 4,320.00 บาท ยอดรวม SO เปลี่ยนจาก 4,815.00 เป็น 4,622.40 (รวม VAT)</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1138,7 +1091,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F3. จัดส่ง (Delivery — Scan Verification) — ADR-009 — ต้องสแกน/กรอก Serial ให้ตรงก่อน Validate เสมอ เหมือน Mode 2</t>
+          <t>E3. จัดส่ง (Delivery — Scan Verification) — ADR-009 — ต้องสแกน/กรอก Serial ให้ตรงก่อน Validate เสมอ ยังใช้ตรรกะเดิม ไม่เปลี่ยนตามกลไกตัดใหม่</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1160,7 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-09</t>
+          <t>TC-E2E-M3-08</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1217,13 +1170,14 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-08 เสร็จแล้ว มีใบส่งของสถานะ Ready รออยู่</t>
+          <t>ทำ TC-E2E-M3-07 เสร็จแล้ว มีใบส่งของสถานะ Ready รออยู่</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิดใบส่งของ (Delivery) ที่เกิดขึ้นอัตโนมัติ
-2. กดปุ่ม Validate ทันทีโดยยังไม่กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial ของแผ่นที่ตัดจริง</t>
+2. ถ้าสถานะยังเป็น "Waiting" ให้กด "Check Availability" ก่อน 1 ครั้ง
+3. กดปุ่ม Validate ทันทีโดยยังไม่กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial ของแผ่นที่ตัดจริง</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1233,7 +1187,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ระบบฟ้อง error สองภาษาทันที: "สแกน Serial ไม่ตรง กรุณาสแกนให้ครบก่อน Validate: BLK-26-0013-2" บันทึกไม่ผ่าน</t>
+          <t>ระบบฟ้อง error สองภาษาทันที: "สแกน Serial ไม่ตรง กรุณาสแกนให้ครบก่อน Validate: BLK-26-0028-1" บันทึกไม่ผ่าน</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1241,11 +1195,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>หมายเหตุ: กันส่งแผ่นผิดให้ลูกค้าโดยไม่ได้ตรวจสอบก่อน (ADR-009) — กลไกเดียวกับ Mode 2</t>
-        </is>
-      </c>
+      <c r="H4" s="7" t="n"/>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
@@ -1254,7 +1204,7 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-10</t>
+          <t>TC-E2E-M3-09</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1264,23 +1214,24 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-09 เสร็จแล้ว (เจอ error มาก่อน)</t>
+          <t>ทำ TC-E2E-M3-08 เสร็จแล้ว (เจอ error มาก่อน)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดบรรทัดในใบส่งของ กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial ของแผ่นที่ตัดจริง
-2. กดปุ่ม Validate อีกครั้ง</t>
+          <t>1. เปิดบรรทัดในใบส่งของ กด "Details"
+2. กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial ของแผ่นที่ตัดจริง แล้วกด Save
+3. กดปุ่ม Validate อีกครั้ง</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Scanned Serial = BLK-26-0013-2</t>
+          <t>Scanned Serial = BLK-26-0028-1</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จ — แผ่นที่ขายหายจากสต็อกที่ขายได้ (Available) แล้ว — ตัวอย่างจริง: EG01/OUT/00052</t>
+          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จ — แผ่นที่ขายหายจากสต็อกที่ขายได้ (Available) แล้ว — ตัวอย่างจริง: EG01/OUT/00079</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1328,7 +1279,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F4. บัญชี (Accounting + Payment) — ออกใบแจ้งหนี้ + รับชำระเงิน + ตรวจรายการบัญชี</t>
+          <t>E4. บัญชี (Accounting + Payment) — ออกใบแจ้งหนี้ + รับชำระเงิน + ตรวจรายการบัญชี</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1348,7 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-11</t>
+          <t>TC-E2E-M3-10</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1407,13 +1358,13 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-10 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M3-09 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Sale Order &gt; กด "Create Invoice"
-2. เลือก "Regular invoice" &gt; Create Draft Invoice
+2. เลือก "Regular invoice" &gt; Create Draft
 3. เปิดใบแจ้งหนี้ &gt; กด Confirm</t>
         </is>
       </c>
@@ -1424,7 +1375,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO หลังตัดแผ่นเสร็จ รวม VAT — ตัวอย่างจริง: INV/2026/00010 (4,622.40 บาท = 4,320.00 ก่อน VAT + VAT 7% 302.40)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO หลังคำนวณราคาใหม่แล้ว (ตัวอย่างจริง: INV/2026/00027, 4,622.40)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1441,7 +1392,7 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-12</t>
+          <t>TC-E2E-M3-11</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1451,12 +1402,12 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-11 เสร็จแล้ว (Invoice = Posted)</t>
+          <t>ทำ TC-E2E-M3-10 เสร็จแล้ว (Invoice = Posted)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบแจ้งหนี้ &gt; กด "Register Payment"
+          <t>1. เปิดใบแจ้งหนี้ &gt; กด "Pay"
 2. ตรวจ/ยืนยันยอดและวิธีชำระ &gt; กด Create Payment</t>
         </is>
       </c>
@@ -1467,7 +1418,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment"/"Paid" (Payment Status) — ตัวอย่างจริง: INV/2026/00010 จบที่สถานะ Posted + In Payment</t>
+          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" — ตัวอย่างจริง: INV/2026/00027 จบที่สถานะ Posted + In Payment</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1484,17 +1435,17 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-13</t>
+          <t>TC-E2E-M3-12</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>ตรวจรายการบัญชีบนใบแจ้งหนี้ (รายได้ + VAT + ลูกหนี้ + COGS)</t>
+          <t>ตรวจรายการบัญชีบนใบแจ้งหนี้ (รายได้ + COGS + VAT + ลูกหนี้)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-11 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M3-10 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -1509,13 +1460,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>เห็นเครดิต Sales Revenue - Cut-to-Order (Mode 3) 4,320.00, เครดิต Output VAT 302.40, เดบิต Trade Receivables 4,622.40 (รวม) ตรงตามยอดใบแจ้งหนี้ พร้อมคู่ COGS/Inventory ที่ระบบแนบมาด้วยอัตโนมัติบนใบแจ้งหนี้ใบเดียวกัน (เดบิต COGS 400.00 / เครดิต Inventory 400.00)
-หมายเหตุชื่อบัญชี: บัญชี COGS ที่ขึ้นชื่อ "COGS - Block Direct Sale (Mode 1)" เป็นบัญชีเดียวกับที่ใช้ทุกโหมดที่ตัดสต็อกจาก Block (ไม่ได้จำกัดเฉพาะโหมด 1) ชื่อบัญชีเป็นเพียงชื่อที่ตั้งไว้ตอนสร้างบัญชีแรกสุด ไม่ใช่ตัวบ่งชี้ประเภทการขาย ไม่ใช่ error</t>
+          <t>เห็น 5 บรรทัดบนใบแจ้งหนี้ใบเดียว: เครดิต "411130 Sales Revenue - Cut-to-Order (Mode 3)" (บัญชีเฉพาะของ Mode 3 ไม่ใช่บัญชีทั่วไป), เดบิต "113110 Inventory" (ตัดออก), เดบิต "511110 COGS - Stone Sales (all modes)", เครดิต Output VAT, เดบิต Trade Receivables — ตัวอย่างจริง INV/2026/00027: รายได้ 4,320.00 / COGS-Inventory คู่ละ 300.00 / VAT 302.40 / ลูกหนี้ 4,622.40 (ยอดรวมสมดุล 4,922.40 = 4,922.40) พร้อม Analytic Distribution ครบ 3 มิติ</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H6" s="7" t="n"/>
@@ -1527,24 +1477,23 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-14</t>
+          <t>TC-E2E-M3-13</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>ตรวจว่าต้นทุนขาย (COGS) ไม่ถูกบันทึกซ้ำ</t>
+          <t>ตรวจว่าไม่มี Journal Entry ซ้ำจากใบส่งของ (ไม่มี COGS ซ้ำ)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-10 เสร็จแล้ว (Delivery = Done) และ TC-E2E-M3-11 เสร็จแล้ว (Invoice = Posted)</t>
+          <t>ทำ TC-E2E-M3-09 เสร็จแล้ว (Delivery = Done)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Accounting &gt; Journal Entries
-2. ค้นหา entry ที่มี Reference ตรงกับเลขที่ใบส่งของ (EG01/OUT/00052)
-3. เทียบกับคู่ COGS/Inventory ที่เห็นใน TC-E2E-M3-13</t>
+2. ค้นหา entry ที่มี Reference ตรงกับเลขที่ใบส่งของ (เช่น EG01/OUT/00079)</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1554,19 +1503,15 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ไม่พบ Journal Entry แยกต่างหากที่อ้างอิงใบส่งของเลย — คู่ COGS/Inventory ที่เห็นใน TC-E2E-M3-13 (ฝังอยู่ในใบแจ้งหนี้) เป็นชุดเดียวที่มีอยู่จริง ไม่ซ้ำ</t>
+          <t>ไม่พบ Journal Entry แยกต่างหากสำหรับใบส่งของนี้เลย (มีเฉพาะ entry ของขั้นตอนตัด/ผลิตซึ่งเป็นคนละเรื่องกัน) — COGS มีบันทึกอยู่ที่เดียวคือในใบแจ้งหนี้ (INV/2026/00027) ไม่มีการนับซ้ำ ยืนยันแล้วว่ากลไกตัดใหม่ (13 ก.ย. 2026) ไม่กระทบพฤติกรรมนี้</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>✅ ยืนยันแล้วจากการรันจริง: ปัญหา COGS บันทึกซ้ำที่เคยพบใน Mode 1/2 (TC-E2E-M1-12 / TC-E2E-M2-12) ไม่เกิดกับการรันนี้ — เพราะรันหลัง ADR-054/055 แก้ไขแล้วในวันเดียวกัน (2026-09-06) ก่อนหน้านี้ Mode 1/2 พบคู่ COGS/Inventory ขึ้นซ้ำสองชุด (ใบแจ้งหนี้ฝังเองชุดหนึ่ง + Journal Entry แยกจากใบส่งของอีกชุด) จากบั๊ก native ของ Odoo ที่แก้ไปแล้ว</t>
-        </is>
-      </c>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>

</xml_diff>

<commit_message>
Archive all 5 Golden Path docs, rebuild Mode 3 (Cut-to-Order) v3
Old Mode 1-5 Golden Path Test Case docs moved to qa/_archive/ (versioned
filenames, assets, and xlsx snapshots) with archived.html/library.html
cross-links updated.

Rebuilt Mode 3 as v3 (15 test cases) reflecting the current batch-cut
mechanism (ADR-066: planned/actual slab lines + yield%) and the guided
banner/"Move to Production" button UI (Session 136-138) — full live
Playwright run on mbx-ee-dev, real fixture (PO P00055 -> Block BLK-26-0030
-> SO S00131 -> MO EG01/STCUT/00044 cutting 2 slabs from 1 block ->
Delivery EG01/OUT/00085 -> Invoice INV/2026/00033).

Mode 5 (also affected by the same UI changes) intentionally deferred.
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode3.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode3.xlsx
@@ -484,14 +484,14 @@
     <row r="5">
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Total test cases: 13</t>
+          <t>Total test cases: 15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 11 / 2 / 0</t>
+          <t>High / Medium / Low: 12 / 3 / 0</t>
         </is>
       </c>
     </row>
@@ -520,11 +520,11 @@
     <row r="10">
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>E2 — ผลิต (Production — ตัด Slab จริง)</t>
+          <t>E2 — ผลิต (Production — ตัด Block→Slab แบบวางแผน/บันทึกจริง)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -717,7 +717,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น Sales Order ยอดรวมคำนวณจากราคาตั้งต้นของสินค้า (ตัวอย่างจริง: S00125, 4,500 + VAT 7% = 4,815.00 บาท) — ราคานี้ยังไม่ใช่ราคาจริง จะคำนวณใหม่อัตโนมัติหลังตัดเสร็จ (ดู TC-E2E-M3-07) มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ แต่ยังส่งไม่ได้เพราะยังไม่มีของจริง</t>
+          <t>SO เปลี่ยนสถานะเป็น Sales Order ยอดรวมคำนวณจากราคาตั้งต้นของสินค้า (ตัวอย่างจริง: S00131, 4,500 + VAT 7% = 4,815.00 บาท) — ราคานี้ยังไม่ใช่ราคาจริง จะคำนวณใหม่อัตโนมัติหลังตัดเสร็จ (ดู TC-E2E-M3-09) มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ แต่ยังส่งไม่ได้เพราะยังไม่มีของจริง</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -765,7 +765,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>E2. ผลิต (Production — ตัด Slab จริง) — กลไกใหม่ 13 ก.ย. 2026 — สร้าง Manufacturing Order ตรงในแอป Manufacturing ไม่ต้องผ่าน wizard แล้ว</t>
+          <t>E2. ผลิต (Production — ตัด Block→Slab แบบวางแผน/บันทึกจริง) — กลไกใหม่ 14 ก.ย.-16 ก.ย. 2026 (ADR-066 + Session 136-138) — วางแผนจำนวนแผ่นอัตโนมัติ, ปุ่ม "ย้ายด่วน", banner นำทาง, บันทึกขนาดจริง+Yield %</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>สร้าง Manufacturing Order ผูกกับ Block และ SO line โดยตรง</t>
+          <t>สร้าง Manufacturing Order ผูกกับ Block และ SO line — ระบบวางแผนจำนวนแผ่นให้อัตโนมัติ</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -857,15 +857,15 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Stone Block = BLK-26-0028
-Target Slab L (M) = 1.2
-Target Slab H (M) = 0.8
-For Sale Order Line = S00125</t>
+          <t>Stone Block = BLK-26-0030
+Target Slab L (M) = 0.80
+Target Slab H (M) = 0.50
+For Sale Order Line = S00131</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>สร้าง Manufacturing Order สำเร็จ ระบบเติม Product และ Bill of Material ให้อัตโนมัติจาก Block ที่เลือก (ตัวอย่างจริง: EG01/STCUT/00042)</t>
+          <t>สร้าง Manufacturing Order สำเร็จ (ตัวอย่างจริง: EG01/STCUT/00044) แท็บ "Planned/Actual Slabs" มี 2 แถวเกิดขึ้นเองอัตโนมัติ (ก้อนนี้ตัดได้ 2 แผ่นจากขนาดที่กรอก) banner สีเหลืองด้านบนแจ้งว่ายังไม่พร้อม Confirm</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>✨ กลไกใหม่ (เปลี่ยน 13 ก.ย. 2026): ไม่มี "Factory Worklist"/"Cut to Order" wizard แล้ว — Admin สร้าง Manufacturing Order ตรงในแอป Manufacturing ได้เลย เลือก Block ที่ช่อง "Stone Block" ระบบจะเติม Product/Bill of Material ให้อัตโนมัติ</t>
+          <t>✨ กลไกใหม่ (เปลี่ยน 14 ก.ย. 2026, ADR-066): เลือก Block + กรอกขนาดที่ต้องการ (Target Slab L/H) แล้วระบบจะคำนวณเองว่าก้อนนี้ตัดได้กี่แผ่น เติมแถว "Planned/Actual Slabs" ให้อัตโนมัติ — ไม่ต้องสร้าง MO ทีละแผ่นแบบเดิมอีกแล้ว</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -911,7 +911,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ระบบฟ้อง error สองภาษาทันที ระบุปริมาณที่ต้องการเทียบกับที่มีอยู่จริงที่สถานีตัด บันทึกไม่ผ่าน — ตัวอย่างจริง: "Block BLK-26-0028 ยังไม่ได้ย้ายไปสถานีตัด (Stone Production) เพียงพอ — ต้องการ 0.019 m³ แต่อยู่ที่สถานีตัดแล้วแค่ 0.000 m³"</t>
+          <t>ระบบฟ้อง error สองภาษาทันที ระบุปริมาณที่ต้องการเทียบกับที่มีอยู่จริงที่สถานีตัด บันทึกไม่ผ่าน — ตัวอย่างจริง: "Block BLK-26-0030 ยังไม่ได้ย้ายไปสถานีตัด (Stone Production) เพียงพอ — ต้องการ 0.016 m³ แต่อยู่ที่สถานีตัดแล้วแค่ 0.000 m³"</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>ย้าย Block ไปสถานีตัด (Internal Transfer)</t>
+          <t>กดปุ่ม "ย้ายด่วน (Move to Production)" — ย้าย Block ในคลิกเดียว</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -943,21 +943,17 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Inventory &gt; Internal Transfers &gt; New
-2. Source Location = Stone Available, Destination Location = Stone Production
-3. เพิ่มสินค้า Block นั้น กรอกจำนวนที่ต้องการย้าย
-4. กด Validate</t>
+          <t>1. กดปุ่ม "ย้ายด่วน (Move to Production)" บน Manufacturing Order</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>สินค้า = E2E Mode3 Fresh Test - Block
-จำนวน = 0.02 m³</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ใบย้ายสถานะเปลี่ยนเป็น Done สำเร็จ — ตัวอย่างจริง: EG01/INT/00058 — Block ก้อนนั้นย้ายไปอยู่ที่ Location "Stone Production" ครบตามจำนวนที่ย้าย</t>
+          <t>แจ้งเตือนสำเร็จทันที — ตัวอย่างจริง: "ย้ายสำเร็จ (Moved). Block BLK-26-0030 ย้ายไป Stone Production แล้ว 0.020 หน่วย — กด Confirm ได้เลย"</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -965,7 +961,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="7" t="n"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>✨ ปุ่มใหม่ (Session 137, 16 ก.ย. 2026): แทนที่การออกไปสร้าง Internal Transfer เองที่เมนู Inventory แล้วต้องย้อนกลับมา — ปุ่มนี้อยู่บน MO เลย ย้าย+ยืนยันใบย้ายให้เสร็จในคลิกเดียว</t>
+        </is>
+      </c>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
@@ -989,8 +989,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1. กลับไปที่ Manufacturing Order เดิม
-2. กดปุ่ม Confirm อีกครั้ง</t>
+          <t>1. กดปุ่ม Confirm อีกครั้ง</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1000,7 +999,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ยืนยันสำเร็จ ไม่มี error แล้ว เพราะ Block ถูกย้ายมาสถานีตัดครบตามจำนวนแล้ว — สถานะเปลี่ยนเป็น Confirmed ปุ่ม "Complete Cut" ปรากฏพร้อมกดขั้นถัดไป</t>
+          <t>ยืนยันสำเร็จ ไม่มี error แล้ว เพราะ Block ถูกย้ายมาสถานีตัดครบตามจำนวนแล้ว — สถานะเปลี่ยนเป็น Confirmed banner สีฟ้าด้านบนแนะนำขั้นตอนถัดไปให้ไปแท็บ "Work Orders"</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1022,7 +1021,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>กด "Complete Cut" — ได้แผ่นจริง ราคา SO คำนวณใหม่อัตโนมัติ</t>
+          <t>ทำ Work Order ให้เสร็จ (Transport + ตัด)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1032,8 +1031,8 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม "Complete Cut" บน Manufacturing Order
-2. กลับไปเปิด Sale Order เดิมดูราคา</t>
+          <t>1. ไปแท็บ "Work Orders"
+2. กดเริ่ม (▶) แต่ละขั้นตอนแล้วกดทำเสร็จตามลำดับจนครบทุกแถว</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1043,12 +1042,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Manufacturing Order เสร็จสมบูรณ์ (สถานะ Done) เกิดแผ่นหินใหม่ 1 แผ่นตามขนาดที่ตัดจริง (Lot/Serial ใหม่) ผูกกับบรรทัด SO เดิมให้อัตโนมัติ ราคาต่อหน่วยของบรรทัด SO เปลี่ยนจากราคาตั้งต้นเป็นราคาจริงตามขนาดที่ตัดได้ทันที — ตัวอย่างจริง: แผ่น BLK-26-0028-1 (1.2×0.8 ม. = 0.96 ตร.ม.) ยอดรวม SO เปลี่ยนจาก 4,815.00 เป็น 4,622.40 (รวม VAT) ทันที เห็นการเปลี่ยนแปลงบันทึกไว้ใน chatter log ของ SO</t>
+          <t>ทุกแถวในแท็บ Work Orders ขึ้นสถานะ "Finished" ครบ (ตัวอย่างจริง: Transport → Gangsaw) MO เปลี่ยนสถานะเป็น "To Close" โดยอัตโนมัติ</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1056,6 +1055,101 @@
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M3-08</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>บันทึกขนาดที่ตัดได้จริงในแท็บ "Planned/Actual Slabs"</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M3-07 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>1. ไปแท็บ "Planned/Actual Slabs"
+2. แก้ไขคอลัมน์ Actual L/H ของแผ่นที่ตัดได้ไม่เท่าแผน (แผ่นอื่นปล่อยตามค่าเริ่มต้นถ้าตัดได้ตรงแผนจริง)</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>แผ่นที่ 1: Actual L = 0.78, Actual H = 0.49 (ของจริงเล็กกว่าแผนนิดหน่อยจากรอยตัด)
+แผ่นที่ 2: Actual L = 0.80, Actual H = 0.50 (ตรงแผนเป๊ะ)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>บันทึกสำเร็จ ผลรวมท้ายแท็บคำนวณใหม่อัตโนมัติ — ตัวอย่างจริง: Planned Total 0.80 ตร.ม. / Actual Total 0.7822 ตร.ม. / Yield 97.78% (ไม่ขึ้น Exception เพราะเบี่ยงเบนไม่ถึง 10%)</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>✨ กลไกใหม่ (ADR-066): แต่ละแผ่นมีคอลัมน์ Actual L/H/Thickness แยกจาก Planned — Factory แก้เฉพาะแผ่นที่ตัดได้ไม่ตรงแผน ระบบคำนวณ Yield % เทียบแผนให้อัตโนมัติที่ท้ายแท็บ</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M3-09</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>กด "Complete Cut" — ได้แผ่นจริง 2 แผ่นจาก 1 ก้อน ราคา SO คำนวณใหม่อัตโนมัติ</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M3-08 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม "Complete Cut" บน Manufacturing Order
+2. กลับไปเปิด Sale Order เดิมดูราคา</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Manufacturing Order เสร็จสมบูรณ์ (สถานะ Done) เกิดแผ่นหินใหม่ 2 แผ่นจากก้อนเดียว (Lot/Serial ใหม่ทั้งคู่) — แผ่นที่ตรงกับความต้องการของบรรทัด SO ถูกจองให้อัตโนมัติ (ตัวอย่างจริง: BLK-26-0030-1, 0.78×0.49 ม.) ส่วนแผ่นที่เหลือค้างเป็นสต็อกว่างขายต่อได้ (BLK-26-0030-2, 0.80×0.50 ม.) ราคาต่อหน่วยของบรรทัด SO เปลี่ยนจากราคาตั้งต้นเป็นราคาจริงตามขนาดที่ตัดได้ทันที — ตัวอย่างจริง: ยอดรวม SO เปลี่ยนจาก 4,815.00 เป็น 1,840.29 (รวม VAT) ทันที เห็นการเปลี่ยนแปลงบันทึกไว้ใน chatter log ของ SO</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>✨ นี่คือจุดเด่นของกลไกใหม่ทั้งหมด: 1 ก้อนตัดได้หลายแผ่นในครั้งเดียว แผ่นที่ SO line ต้องการถูกจองอัตโนมัติ ส่วนแผ่นที่เหลือเก็บเป็นสต็อกส่วนเกินไว้ขายต่อ</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="L10" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1160,7 +1254,7 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-08</t>
+          <t>TC-E2E-M3-10</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1170,14 +1264,13 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-07 เสร็จแล้ว มีใบส่งของสถานะ Ready รออยู่</t>
+          <t>ทำ TC-E2E-M3-09 เสร็จแล้ว มีใบส่งของสถานะ Ready รออยู่</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิดใบส่งของ (Delivery) ที่เกิดขึ้นอัตโนมัติ
-2. ถ้าสถานะยังเป็น "Waiting" ให้กด "Check Availability" ก่อน 1 ครั้ง
-3. กดปุ่ม Validate ทันทีโดยยังไม่กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial ของแผ่นที่ตัดจริง</t>
+2. กดปุ่ม Validate ทันทีโดยยังไม่กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial ของแผ่นที่ตัดจริง</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1187,7 +1280,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ระบบฟ้อง error สองภาษาทันที: "สแกน Serial ไม่ตรง กรุณาสแกนให้ครบก่อน Validate: BLK-26-0028-1" บันทึกไม่ผ่าน</t>
+          <t>ระบบฟ้อง error สองภาษาทันที: "สแกน Serial ไม่ตรง กรุณาสแกนให้ครบก่อน Validate: BLK-26-0030-1" บันทึกไม่ผ่าน</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1204,7 +1297,7 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-09</t>
+          <t>TC-E2E-M3-11</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1214,7 +1307,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-08 เสร็จแล้ว (เจอ error มาก่อน)</t>
+          <t>ทำ TC-E2E-M3-10 เสร็จแล้ว (เจอ error มาก่อน)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -1226,12 +1319,12 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Scanned Serial = BLK-26-0028-1</t>
+          <t>Scanned Serial = BLK-26-0030-1</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จ — แผ่นที่ขายหายจากสต็อกที่ขายได้ (Available) แล้ว — ตัวอย่างจริง: EG01/OUT/00079</t>
+          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จ — แผ่นที่ขายหายจากสต็อกที่ขายได้ (Available) แล้ว — ตัวอย่างจริง: EG01/OUT/00085</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1348,7 +1441,7 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-10</t>
+          <t>TC-E2E-M3-12</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1358,7 +1451,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-09 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M3-11 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -1375,7 +1468,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO หลังคำนวณราคาใหม่แล้ว (ตัวอย่างจริง: INV/2026/00027, 4,622.40)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO หลังคำนวณราคาใหม่แล้ว (ตัวอย่างจริง: INV/2026/00033, 1,840.29)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1392,7 +1485,7 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-11</t>
+          <t>TC-E2E-M3-13</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1402,7 +1495,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-10 เสร็จแล้ว (Invoice = Posted)</t>
+          <t>ทำ TC-E2E-M3-12 เสร็จแล้ว (Invoice = Posted)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -1418,7 +1511,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" — ตัวอย่างจริง: INV/2026/00027 จบที่สถานะ Posted + In Payment</t>
+          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" — ตัวอย่างจริง: INV/2026/00033 จบที่สถานะ Posted + In Payment</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1435,7 +1528,7 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-12</t>
+          <t>TC-E2E-M3-14</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -1445,12 +1538,12 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-10 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M3-12 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Customer Invoice &gt; กด smart button "Journal Items"</t>
+          <t>1. เปิด Customer Invoice &gt; กด แท็บ "Journal Items"</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1460,7 +1553,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>เห็น 5 บรรทัดบนใบแจ้งหนี้ใบเดียว: เครดิต "411130 Sales Revenue - Cut-to-Order (Mode 3)" (บัญชีเฉพาะของ Mode 3 ไม่ใช่บัญชีทั่วไป), เดบิต "113110 Inventory" (ตัดออก), เดบิต "511110 COGS - Stone Sales (all modes)", เครดิต Output VAT, เดบิต Trade Receivables — ตัวอย่างจริง INV/2026/00027: รายได้ 4,320.00 / COGS-Inventory คู่ละ 300.00 / VAT 302.40 / ลูกหนี้ 4,622.40 (ยอดรวมสมดุล 4,922.40 = 4,922.40) พร้อม Analytic Distribution ครบ 3 มิติ</t>
+          <t>เห็น 5 บรรทัดบนใบแจ้งหนี้ใบเดียว: เครดิต "411130 Sales Revenue - Cut-to-Order (Mode 3)" (บัญชีเฉพาะของ Mode 3 ไม่ใช่บัญชีทั่วไป), เครดิต "113110 Inventory" (ตัดออก), เดบิต "511110 COGS - Stone Sales (all modes)", เครดิต Output VAT, เดบิต Trade Receivables — ตัวอย่างจริง INV/2026/00033: รายได้ 1,719.90 / Inventory-COGS คู่ละ 150.00 / VAT 120.39 / ลูกหนี้ 1,840.29 (ยอดรวมสมดุล 1,990.29 = 1,990.29) พร้อม Analytic Distribution ครบ 3 มิติ (Material/Block/หมวดวัสดุ)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1477,7 +1570,7 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M3-13</t>
+          <t>TC-E2E-M3-15</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1487,13 +1580,13 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M3-09 เสร็จแล้ว (Delivery = Done)</t>
+          <t>ทำ TC-E2E-M3-11 เสร็จแล้ว (Delivery = Done)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Accounting &gt; Journal Entries
-2. ค้นหา entry ที่มี Reference ตรงกับเลขที่ใบส่งของ (เช่น EG01/OUT/00079)</t>
+2. ค้นหา entry ที่มี Reference ตรงกับเลขที่ใบส่งของ (เช่น EG01/OUT/00085)</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1503,7 +1596,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ไม่พบ Journal Entry แยกต่างหากสำหรับใบส่งของนี้เลย (มีเฉพาะ entry ของขั้นตอนตัด/ผลิตซึ่งเป็นคนละเรื่องกัน) — COGS มีบันทึกอยู่ที่เดียวคือในใบแจ้งหนี้ (INV/2026/00027) ไม่มีการนับซ้ำ ยืนยันแล้วว่ากลไกตัดใหม่ (13 ก.ย. 2026) ไม่กระทบพฤติกรรมนี้</t>
+          <t>ไม่พบ Journal Entry แยกต่างหากสำหรับใบส่งของนี้เลย (มีเฉพาะ entry ของขั้นตอนตัด/ผลิตซึ่งเป็นคนละเรื่องกัน) — COGS มีบันทึกอยู่ที่เดียวคือในใบแจ้งหนี้ (INV/2026/00033) ไม่มีการนับซ้ำ ยืนยันแล้วว่ากลไกตัดแบบวางแผน/บันทึกจริง (16 ก.ย. 2026) ไม่กระทบพฤติกรรมนี้</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">

</xml_diff>